<commit_message>
added correct homework file
</commit_message>
<xml_diff>
--- a/homework1.xlsx
+++ b/homework1.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DataAnalytics\pre-week-2\homework1.xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DataAnalytics\pre-week-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AC87FA9-8F39-48FD-9920-237AC567FD5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47594C46-B0CE-4F90-87D6-619CAB30E43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="8170" xr2:uid="{E6E81B3A-2E10-459D-8309-3FB902560461}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E6E81B3A-2E10-459D-8309-3FB902560461}"/>
   </bookViews>
   <sheets>
     <sheet name="Store_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Store_summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -669,13 +670,24 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="28" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.35"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6AA43DF-DB38-4B31-80C5-B35AF1B7ADE0}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>